<commit_message>
Updated GBR model - 2025-11-04 10:50
</commit_message>
<xml_diff>
--- a/VerveStacks_GBR/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_GBR/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GBR\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A4A1634-9138-495D-8138-5AD5FECD63E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{33BBCEE1-7978-4472-962D-56AC43EF03FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6129,7 +6129,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76FA3472-5162-45D2-951D-C33600802E57}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69D80AF8-A639-4149-8EE8-CEE52A16E04B}">
   <dimension ref="B9:M31"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6917,7 +6917,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{538C6587-AA9D-4C6C-9C78-6528B03A7B91}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB701B0C-1075-46D6-BEA8-B372A30D5AB1}">
   <dimension ref="B9:Z44"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8892,7 +8892,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45AB5CB7-04B8-4FC5-ABB8-3CFADB2AF8DE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8FAA95B-5344-43CD-8EA7-8D2C4624CAFE}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated GBR model - 2025-11-06 16:57
</commit_message>
<xml_diff>
--- a/VerveStacks_GBR/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_GBR/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GBR\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{33BBCEE1-7978-4472-962D-56AC43EF03FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1345FFCD-7853-4FC2-96DA-E040516E1891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6129,7 +6129,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69D80AF8-A639-4149-8EE8-CEE52A16E04B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9482183-ABF0-4BA3-8110-B47803D29EEF}">
   <dimension ref="B9:M31"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6917,7 +6917,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB701B0C-1075-46D6-BEA8-B372A30D5AB1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C5F3A98-9FC2-4C8F-BEC6-833F03EB51C5}">
   <dimension ref="B9:Z44"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8892,7 +8892,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8FAA95B-5344-43CD-8EA7-8D2C4624CAFE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC6BEBB3-2BC6-4E87-9FC2-37177E98AC43}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated GBR model - 2025-11-10 16:48
</commit_message>
<xml_diff>
--- a/VerveStacks_GBR/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_GBR/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GBR\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1345FFCD-7853-4FC2-96DA-E040516E1891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D3E952F-E70C-412F-B698-DF8C6B56E797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6129,7 +6129,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9482183-ABF0-4BA3-8110-B47803D29EEF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18189517-637A-4281-A84B-4DA48421F637}">
   <dimension ref="B9:M31"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6917,7 +6917,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C5F3A98-9FC2-4C8F-BEC6-833F03EB51C5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{570B617B-0352-41F0-A94E-F2788C8E8D9A}">
   <dimension ref="B9:Z44"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8892,7 +8892,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC6BEBB3-2BC6-4E87-9FC2-37177E98AC43}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00831F3E-912E-4D17-BDA5-0581DA50CC70}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated GBR model - 2025-11-10 17:19
</commit_message>
<xml_diff>
--- a/VerveStacks_GBR/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
+++ b/VerveStacks_GBR/SubRES_Tmpl/SubRES_New_RE_and_Conventional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_GBR\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7D3E952F-E70C-412F-B698-DF8C6B56E797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{191CB024-0F5D-4F1C-8AEC-9D77B51A43AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6129,7 +6129,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18189517-637A-4281-A84B-4DA48421F637}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80918EC1-9369-401B-9091-8078F113000E}">
   <dimension ref="B9:M31"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -6917,7 +6917,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{570B617B-0352-41F0-A94E-F2788C8E8D9A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C26B8568-4CEE-4AE4-9D76-C043E65090C3}">
   <dimension ref="B9:Z44"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -8892,7 +8892,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00831F3E-912E-4D17-BDA5-0581DA50CC70}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{007837AB-2FA8-4280-956C-1183F83CFA4B}">
   <dimension ref="B9:P73"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>